<commit_message>
fix: update fetching script and rank distribution
</commit_message>
<xml_diff>
--- a/src/ANALYSIS/LoL Rank Distribution via DPM.LOL.xlsx
+++ b/src/ANALYSIS/LoL Rank Distribution via DPM.LOL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HARDPC\Desktop\github\riotdev\src\ANALYSIS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B53C2A8D-AA8C-4441-B7EF-161606B09EC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{821E83A1-EF07-4A4C-80B3-A0E43A94484E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{A0029291-6BCC-4475-BEED-018B6CE89298}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{A0029291-6BCC-4475-BEED-018B6CE89298}"/>
   </bookViews>
   <sheets>
     <sheet name="Server_sampling" sheetId="7" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1653" uniqueCount="608">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1654" uniqueCount="608">
   <si>
     <t>Tier</t>
   </si>
@@ -1954,7 +1954,7 @@
     <tableColumn id="4" xr3:uid="{7253E19C-8CB6-4910-96EE-75B508160C51}" name="Amount">
       <calculatedColumnFormula>I30</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{321DB45C-0D15-47B1-B19B-72BCB1455078}" name="%" dataDxfId="0">
+    <tableColumn id="5" xr3:uid="{321DB45C-0D15-47B1-B19B-72BCB1455078}" name="%" dataDxfId="4">
       <calculatedColumnFormula>(O10/$L$10*100)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{7126E4C5-DCAF-43BA-B1F2-F4B5C8F16D7C}" name="Fetch amount"/>
@@ -1974,7 +1974,7 @@
     <tableColumn id="4" xr3:uid="{E3C604EC-F001-4617-AFA3-15766EEDDF78}" name="Amount">
       <calculatedColumnFormula>I30</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{A75305CC-1838-48D2-BB09-F3FA864F5D92}" name="%" dataDxfId="4">
+    <tableColumn id="5" xr3:uid="{A75305CC-1838-48D2-BB09-F3FA864F5D92}" name="%" dataDxfId="3">
       <calculatedColumnFormula>(O10/$L$10*100)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{29B232FD-1B51-4610-A16A-CE07A56320AF}" name="Fetch amount"/>
@@ -1994,7 +1994,7 @@
     <tableColumn id="4" xr3:uid="{82900B8D-8D90-4B9A-86C7-B8CA92859808}" name="Amount">
       <calculatedColumnFormula>I30</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{34769021-C164-4382-82C5-16F0A20A9E2B}" name="%" dataDxfId="3">
+    <tableColumn id="5" xr3:uid="{34769021-C164-4382-82C5-16F0A20A9E2B}" name="%" dataDxfId="2">
       <calculatedColumnFormula>(O10/$L$10*100)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{92057921-7202-4155-A3DC-2E13A232A4A7}" name="Fetch amount"/>
@@ -2014,7 +2014,7 @@
     <tableColumn id="4" xr3:uid="{8A105A44-B3B8-419F-8B3E-1CB1AE0C6C85}" name="Amount">
       <calculatedColumnFormula>I30</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{4B52B8BE-0230-4E4B-85B3-1CB310770D9D}" name="%" dataDxfId="2">
+    <tableColumn id="5" xr3:uid="{4B52B8BE-0230-4E4B-85B3-1CB310770D9D}" name="%" dataDxfId="1">
       <calculatedColumnFormula>(O10/$L$10*100)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{61145AFE-EEBC-43B5-B245-7F0779585748}" name="Fetch amount"/>
@@ -2034,7 +2034,7 @@
     <tableColumn id="4" xr3:uid="{FF8A68C3-5811-4ECA-97CE-F0B4A7EB663A}" name="Amount">
       <calculatedColumnFormula>I30</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{A65878B4-1590-4844-95F0-53A9CD6A82DD}" name="%" dataDxfId="1">
+    <tableColumn id="5" xr3:uid="{A65878B4-1590-4844-95F0-53A9CD6A82DD}" name="%" dataDxfId="0">
       <calculatedColumnFormula>(O10/$L$10*100)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{A2B05F9B-3C0D-4515-ABCC-07C1F135992D}" name="Fetch amount"/>
@@ -4183,7 +4183,7 @@
         <v>15.0739563421595</v>
       </c>
       <c r="Q11">
-        <f t="shared" ref="Q11:Q19" si="1">INT($M$10*(P11/100))</f>
+        <f t="shared" ref="Q11:Q17" si="1">INT($M$10*(P11/100))</f>
         <v>422</v>
       </c>
     </row>
@@ -7792,6 +7792,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7820,8 +7821,8 @@
       <c r="H1" t="s">
         <v>1</v>
       </c>
-      <c r="I1">
-        <v>15000</v>
+      <c r="I1" t="s">
+        <v>602</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
@@ -9114,23 +9115,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="5c371023-5351-4a2c-b274-12e7bf1d720d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010004DC25A874A6A34FA57A1410CFDC29AE" ma:contentTypeVersion="10" ma:contentTypeDescription="Utwórz nowy dokument." ma:contentTypeScope="" ma:versionID="d2e102214b3071d241a3f49a1e8f5f14">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="5c371023-5351-4a2c-b274-12e7bf1d720d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="391f2fa415d308e115475a881a25dbb9" ns3:_="">
     <xsd:import namespace="5c371023-5351-4a2c-b274-12e7bf1d720d"/>
@@ -9312,31 +9296,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5AE49221-E7C8-41E3-8922-F3E2B4173845}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="5c371023-5351-4a2c-b274-12e7bf1d720d"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBC685B8-DEF0-4295-9DEC-106CE61F28BC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="5c371023-5351-4a2c-b274-12e7bf1d720d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D8FEF492-466C-4B24-8828-667CE88459D8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9352,4 +9329,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBC685B8-DEF0-4295-9DEC-106CE61F28BC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5AE49221-E7C8-41E3-8922-F3E2B4173845}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="5c371023-5351-4a2c-b274-12e7bf1d720d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>